<commit_message>
Update database requirements coverage after SQL validation
Update DATA-001 through DATA-008 with local SQL validation evidence, coverage status, execution status and remaining limitations.
</commit_message>
<xml_diff>
--- a/requirements-traceability/booking-system-requirements-traceability-matrix.xlsx
+++ b/requirements-traceability/booking-system-requirements-traceability-matrix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Career-Reentry-Portfolio\Day-3-Test-Coverage-Traceability-Defects\Traceability-Matrix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Career-Reentry-Portfolio\Day-4-PostgreSQL-Database-Testing\Updated-Traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D0CD9F-D58C-4761-AEFE-8A52507D7E8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3CCAA0-5EC8-43D0-AD47-10C9C39F69A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2715" yWindow="3015" windowWidth="22785" windowHeight="15345" xr2:uid="{2EB850F2-E74B-4566-842F-107018F40829}"/>
+    <workbookView xWindow="705" yWindow="2445" windowWidth="22785" windowHeight="15345" xr2:uid="{2EB850F2-E74B-4566-842F-107018F40829}"/>
   </bookViews>
   <sheets>
     <sheet name="Traceability_Matrix" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="157">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -374,90 +374,54 @@
     <t>Store every successfully created booking in the database</t>
   </si>
   <si>
-    <t>Planned for SQL testing</t>
-  </si>
-  <si>
     <t>Planned</t>
   </si>
   <si>
-    <t>Database validation begins on Day 4</t>
-  </si>
-  <si>
     <t>DATA-002</t>
   </si>
   <si>
     <t>Ensure API booking data matches the corresponding database record</t>
   </si>
   <si>
-    <t>Planned for API and SQL testing</t>
-  </si>
-  <si>
-    <t>Requires API and database comparison</t>
-  </si>
-  <si>
     <t>DATA-003</t>
   </si>
   <si>
     <t>Store a unique identifier for every booking</t>
   </si>
   <si>
-    <t>TC-BOOK-001; Planned SQL validation</t>
-  </si>
-  <si>
     <t>Partially Covered</t>
   </si>
   <si>
-    <t>API ID test created; database uniqueness test pending</t>
-  </si>
-  <si>
     <t>DATA-004</t>
   </si>
   <si>
     <t>Connect every booking to a valid customer record</t>
   </si>
   <si>
-    <t>Foreign-key validation pending</t>
-  </si>
-  <si>
     <t>DATA-005</t>
   </si>
   <si>
     <t>Prevent null values in required database fields</t>
   </si>
   <si>
-    <t>Null-validation queries pending</t>
-  </si>
-  <si>
     <t>DATA-006</t>
   </si>
   <si>
     <t>Store checkout dates later than check-in dates</t>
   </si>
   <si>
-    <t>TC-BOOK-004; TC-UPD-005; Planned SQL validation</t>
-  </si>
-  <si>
-    <t>API cases created; database validation pending</t>
-  </si>
-  <si>
     <t>DATA-007</t>
   </si>
   <si>
     <t>Store a total booking price greater than zero</t>
   </si>
   <si>
-    <t>TC-BOOK-005; TC-VAL-001; TC-VAL-002; Planned SQL validation</t>
-  </si>
-  <si>
     <t>DATA-008</t>
   </si>
   <si>
     <t>Remove or deactivate a booking after successful deletion</t>
   </si>
   <si>
-    <t>TC-DEL-001; TC-DEL-002; Planned SQL validation</t>
-  </si>
-  <si>
     <t>NFR-001</t>
   </si>
   <si>
@@ -498,6 +462,54 @@
   </si>
   <si>
     <t>Ongoing process control; secret scanning to be added later</t>
+  </si>
+  <si>
+    <t>SQL-VAL-01; SQL-VAL-02</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Local schema population and stored booking records were validated. Direct API persistence remains pending because the local database is not the demonstration API database.</t>
+  </si>
+  <si>
+    <t>Planned for future API-to-database testing</t>
+  </si>
+  <si>
+    <t>Direct API-to-database comparison is unavailable because the local portfolio database is not the database behind the demonstration API.</t>
+  </si>
+  <si>
+    <t>SQL-VAL-05</t>
+  </si>
+  <si>
+    <t>Booking identifier uniqueness was validated in the local portfolio database. No duplicate booking identifier groups were detected.</t>
+  </si>
+  <si>
+    <t>SQL-VAL-10; SQL-CON-04</t>
+  </si>
+  <si>
+    <t>No orphan bookings were detected, and the foreign-key constraint rejected a booking associated with an unknown customer.</t>
+  </si>
+  <si>
+    <t>SQL-VAL-07; SQL-CON-01; SQL-CON-03</t>
+  </si>
+  <si>
+    <t>Production booking dates were valid, controlled staging date issues were detected, and an invalid booking-date sequence was rejected by the database constraint.</t>
+  </si>
+  <si>
+    <t>SQL-VAL-08; SQL-VAL-14; SQL-CON-05</t>
+  </si>
+  <si>
+    <t>SQL-VAL-09; SQL-VAL-15; SQL-CON-06</t>
+  </si>
+  <si>
+    <t>Production booking prices were positive, controlled staging price issues were detected, and a zero-price booking was rejected by the database constraint.</t>
+  </si>
+  <si>
+    <t>Planned for API deletion and database-verification testing</t>
+  </si>
+  <si>
+    <t>Database verification after an API booking deletion remains pending because the local portfolio database is not connected to the demonstration API.</t>
   </si>
 </sst>
 </file>
@@ -533,11 +545,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,17 +600,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{13DDA59B-61DB-4819-85F2-02EDA509AFA8}" name="Table2" displayName="Table2" ref="A1:H36" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{13DDA59B-61DB-4819-85F2-02EDA509AFA8}" name="Table2" displayName="Table2" ref="A1:H36" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:H36" xr:uid="{13DDA59B-61DB-4819-85F2-02EDA509AFA8}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{0696F431-FE64-4C6F-ABB9-1E5C8418D8D7}" name="Requirement ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{985C1953-F99C-4BF1-BDD1-69B61DEE0E89}" name="Requirement Category" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{E090DE95-2A39-4EDC-A3A7-72EE128A12EF}" name="Requirement Summary" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{0D7BF022-B0A0-41B6-A820-110001CB949F}" name="Linked Test Case IDs" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{9F1C1E61-551C-45D9-B4B4-C8FF18DDD898}" name="Coverage Status" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{4E3AA38E-2BF5-401E-BBEA-4779F82343EC}" name="Execution Status" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{4C973E1F-4C69-44E0-A2F9-400E4723CE4B}" name="Related Defect IDs" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{E76044CA-136A-446D-8381-D19F18320E5E}" name="Comments" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{0696F431-FE64-4C6F-ABB9-1E5C8418D8D7}" name="Requirement ID" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{985C1953-F99C-4BF1-BDD1-69B61DEE0E89}" name="Requirement Category" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{E090DE95-2A39-4EDC-A3A7-72EE128A12EF}" name="Requirement Summary" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{0D7BF022-B0A0-41B6-A820-110001CB949F}" name="Linked Test Case IDs" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{9F1C1E61-551C-45D9-B4B4-C8FF18DDD898}" name="Coverage Status" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{4E3AA38E-2BF5-401E-BBEA-4779F82343EC}" name="Execution Status" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{4C973E1F-4C69-44E0-A2F9-400E4723CE4B}" name="Related Defect IDs" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{E76044CA-136A-446D-8381-D19F18320E5E}" name="Comments" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1535,268 +1548,268 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="F27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1" t="s">
+      <c r="D28" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="B29" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="D29" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="C30" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="D30" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1" t="s">
+      <c r="B31" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="D31" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B32" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D32" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="1"/>
+      <c r="F33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="2"/>
       <c r="H33" s="1" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct DATA-005 traceability comment
Replace the incorrect booking-date comment with the required-field validation evidence for DATA-005.
</commit_message>
<xml_diff>
--- a/requirements-traceability/booking-system-requirements-traceability-matrix.xlsx
+++ b/requirements-traceability/booking-system-requirements-traceability-matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Career-Reentry-Portfolio\Day-4-PostgreSQL-Database-Testing\Updated-Traceability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3CCAA0-5EC8-43D0-AD47-10C9C39F69A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492FCE54-F7A8-4383-ADE2-FB221D533CDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="2445" windowWidth="22785" windowHeight="15345" xr2:uid="{2EB850F2-E74B-4566-842F-107018F40829}"/>
+    <workbookView xWindow="705" yWindow="0" windowWidth="25185" windowHeight="20985" xr2:uid="{2EB850F2-E74B-4566-842F-107018F40829}"/>
   </bookViews>
   <sheets>
     <sheet name="Traceability_Matrix" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="158">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -510,6 +510,9 @@
   </si>
   <si>
     <t>Database verification after an API booking deletion remains pending because the local portfolio database is not connected to the demonstration API.</t>
+  </si>
+  <si>
+    <t>Required production customer fields were validated. Blank first-name and missing last-name records were rejected by database constraints.</t>
   </si>
 </sst>
 </file>
@@ -545,12 +548,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1549,193 +1551,185 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+      <c r="A26" t="s">
         <v>108</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" t="s">
         <v>109</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" t="s">
         <v>141</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" t="s">
         <v>116</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" t="s">
         <v>142</v>
       </c>
-      <c r="G26" s="2"/>
       <c r="H26" s="1" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+      <c r="A27" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" t="s">
         <v>113</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" t="s">
         <v>144</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" t="s">
         <v>111</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="2"/>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
       <c r="H27" s="1" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="A28" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" t="s">
         <v>115</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" t="s">
         <v>146</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F28" s="2" t="s">
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" t="s">
         <v>142</v>
       </c>
-      <c r="G28" s="2"/>
       <c r="H28" s="1" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+      <c r="A29" t="s">
         <v>117</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" t="s">
         <v>109</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" t="s">
         <v>118</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" t="s">
         <v>148</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F29" s="2" t="s">
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
         <v>142</v>
       </c>
-      <c r="G29" s="2"/>
       <c r="H29" s="1" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+      <c r="A30" t="s">
         <v>119</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" t="s">
         <v>109</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" t="s">
         <v>120</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" t="s">
         <v>150</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="2" t="s">
+      <c r="E30" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" t="s">
         <v>142</v>
       </c>
-      <c r="G30" s="2"/>
       <c r="H30" s="1" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+      <c r="A31" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" t="s">
         <v>109</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" t="s">
         <v>122</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" t="s">
         <v>152</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F31" s="2" t="s">
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" t="s">
         <v>142</v>
       </c>
-      <c r="G31" s="2"/>
       <c r="H31" s="1" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="A32" t="s">
         <v>123</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" t="s">
         <v>109</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" t="s">
         <v>124</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" t="s">
         <v>153</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F32" s="2" t="s">
+      <c r="E32" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" t="s">
         <v>142</v>
       </c>
-      <c r="G32" s="2"/>
       <c r="H32" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="A33" t="s">
         <v>125</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" t="s">
         <v>109</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" t="s">
         <v>126</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" t="s">
         <v>155</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" t="s">
         <v>111</v>
       </c>
-      <c r="F33" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="2"/>
+      <c r="F33" t="s">
+        <v>13</v>
+      </c>
       <c r="H33" s="1" t="s">
         <v>156</v>
       </c>

</xml_diff>